<commit_message>
Move the fitness multiplier out of simulateRace and into the spreadsheet
fitScale was `0.8 + 0.2 × fitness/100`, a literal in the simulator. GDD §5.2
marks it ⚖️ and D13 is about to change it, and a constant buried in the race
loop is not tunable — so it becomes fitScaleBase and fitScaleCoef in the
Assumptions sheet, at the same values.

No behaviour change: the golden snapshot is byte-identical.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y6WnxkiCvUQSwseLwaE4jG
</commit_message>
<xml_diff>
--- a/design/space_dog_racing_economy.xlsx
+++ b/design/space_dog_racing_economy.xlsx
@@ -876,7 +876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:D72"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="42" customWidth="1" style="43" min="1" max="1"/>
@@ -1649,144 +1649,181 @@
           <t>Race simulation (GDD §6.2 — the v2 rebalance, 11 September 2026)</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="43" t="inlineStr">
         <is>
           <t>Rebalanced so all four stats matter: measured +10-to-one-stat win rates move from speed 28.8 / stam 16.7 / accel 14.4 / trap 14.0 to rating-weight order, and track length starts to matter at all. D12.</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="43" t="inlineStr">
         <is>
           <t>Race: base speed (m/s)</t>
         </is>
       </c>
-      <c r="B60" t="n">
+      <c r="B60" s="43" t="n">
         <v>13.75</v>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="43" t="inlineStr">
         <is>
           <t>Was 13. The floor every dog runs at before its Speed stat</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="43" t="inlineStr">
         <is>
           <t>Race: speed coefficient (m/s per 100 Speed)</t>
         </is>
       </c>
-      <c r="B61" t="n">
+      <c r="B61" s="43" t="n">
         <v>4.5</v>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="43" t="inlineStr">
         <is>
           <t>Was 6. Cutting this is what stops the race being a pure Speed contest</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="43" t="inlineStr">
         <is>
           <t>Race: fade penalty past the stamina point</t>
         </is>
       </c>
-      <c r="B62" t="n">
+      <c r="B62" s="43" t="n">
         <v>0.5</v>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="43" t="inlineStr">
         <is>
           <t>Was 0.35. Makes Stamina the second-biggest stat, and biggest on a stayer</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="43" t="inlineStr">
         <is>
           <t>Race: acceleration base (m/s²)</t>
         </is>
       </c>
-      <c r="B63" t="n">
+      <c r="B63" s="43" t="n">
         <v>2</v>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="43" t="inlineStr">
         <is>
           <t>Was 4. Less free acceleration, so the stat buys more</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="43" t="inlineStr">
         <is>
           <t>Race: acceleration coefficient (m/s² per 100 Accel)</t>
         </is>
       </c>
-      <c r="B64" t="n">
+      <c r="B64" s="43" t="n">
         <v>5.5</v>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="43" t="inlineStr">
         <is>
           <t>Was 6. Accel now peaks on the 350 m sprints</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="43" t="inlineStr">
         <is>
           <t>Race: break from the boxes (metres at 100 Trap)</t>
         </is>
       </c>
-      <c r="B65" t="n">
+      <c r="B65" s="43" t="n">
         <v>7</v>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="43" t="inlineStr">
         <is>
           <t>Was 3. Trap craft has to be worth something out of the gate</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="43" t="inlineStr">
         <is>
           <t>Race: bump chance on a bend</t>
         </is>
       </c>
-      <c r="B66" t="n">
+      <c r="B66" s="43" t="n">
         <v>0.3</v>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="43" t="inlineStr">
         <is>
           <t>Was 0.10. The other half of what Trap buys</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="43" t="inlineStr">
         <is>
           <t>Race: bump speed penalty</t>
         </is>
       </c>
-      <c r="B67" t="n">
+      <c r="B67" s="43" t="n">
         <v>0.3</v>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C67" s="43" t="inlineStr">
         <is>
           <t>Was 0.15</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" s="43" t="inlineStr">
         <is>
           <t>Race: bump distance (metres)</t>
         </is>
       </c>
-      <c r="B68" t="n">
+      <c r="B68" s="43" t="n">
         <v>1.2</v>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="43" t="inlineStr">
         <is>
           <t>Was 0.6. Dogs this close on a bend may clash</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="87" t="inlineStr">
+        <is>
+          <t>Condition (GDD §5.2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Fitness multiplier: floor</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>fitScale = floor + range x fitness/100, applied to every stat in the race, at every fitness</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Fitness multiplier: range</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Was a literal in simulateRace.ts until v2 Phase A. D13 softens these to 0.90 / 0.10</t>
         </is>
       </c>
     </row>

</xml_diff>